<commit_message>
R1. Corrected report with missing output table
</commit_message>
<xml_diff>
--- a/package-output-map.xlsx
+++ b/package-output-map.xlsx
@@ -1,77 +1,47 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/floswald/git/JPEtemplate/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067DD2C7-24FE-2447-A5A8-8F6542C7C06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="21900" windowHeight="12060" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
-  <si>
-    <t>Data Preparation Program</t>
-  </si>
-  <si>
-    <t>Dataset created</t>
-  </si>
-  <si>
-    <t>Reproduced?</t>
-  </si>
-  <si>
-    <t>Figure/Table #</t>
-  </si>
-  <si>
-    <t>Program</t>
-  </si>
-  <si>
-    <t>Line Number</t>
-  </si>
-  <si>
-    <t>In-text numbers</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
+      <name val="Calibri"/>
+      <charset val="1"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <charset val="1"/>
+      <family val="2"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+    </font>
+    <font>
       <name val="Calibri"/>
+      <charset val="1"/>
       <family val="2"/>
-      <charset val="1"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -90,30 +60,89 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -433,79 +462,732 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M33"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="23.5" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13" customWidth="1"/>
-    <col min="5" max="5" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.5" bestFit="1" customWidth="1"/>
+    <col width="23.44140625" customWidth="1" min="1" max="1"/>
+    <col width="26.5546875" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12.109375" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="44.5546875" customWidth="1" min="6" max="6"/>
+    <col width="11.109375" bestFit="1" customWidth="1" min="7" max="7"/>
+    <col width="11.44140625" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col width="13.44140625" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="7.6640625" bestFit="1" customWidth="1" min="11" max="11"/>
+    <col width="11.109375" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="11.44140625" bestFit="1" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="3"/>
-      <c r="B4" s="3"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Data Preparation Program</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Dataset created</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Reproduced?</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Figure/Table #</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Line Number</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Reproduced?</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>In-text numbers</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Program</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Line Number</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Reproduced?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Table 1</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>2</v>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Table 2</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>201</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Table 3</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>474</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Table 4</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>539</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Table 5</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>680</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Table A1</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>809</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="3" t="n"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Table A2</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>848</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="3" t="n"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Table A3</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1004</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Table A4</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1179</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n"/>
+      <c r="B11" s="3" t="n"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Table A5</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1275</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Table A6</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Table A7</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1552</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Table A8</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>gen_tables.R</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1798</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Figure 1</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>147</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Figure 2</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>184</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Figure 3</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>375</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Figure 4</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>540</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Figure 5</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>573</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Figure 6</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>635</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Figure A1</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>695</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Figure A2</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>788</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Figure A3</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>838</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Figure A4</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>907</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Figure A5</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>936</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Figure A6</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>1004</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Figure A7</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>1074</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Figure A8</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>1131</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Figure A9</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>1191</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Figure A10</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>1227</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Figure A11</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>1273</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Figure A12</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>1371</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Figure A13</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>gen_figures.R</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>1400</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>